<commit_message>
Sold 3 HW THs
</commit_message>
<xml_diff>
--- a/inventory/Inventory.xlsx
+++ b/inventory/Inventory.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" firstSheet="2" activeTab="5"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" firstSheet="2" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Hot Wheels Mainline" sheetId="1" r:id="rId1"/>
@@ -5049,7 +5049,7 @@
         <v>699</v>
       </c>
       <c r="J2" s="18" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="K2" s="18" t="s">
         <v>10</v>
@@ -5084,7 +5084,7 @@
         <v>899</v>
       </c>
       <c r="J3" s="18" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="K3" s="18" t="s">
         <v>10</v>
@@ -5154,7 +5154,7 @@
         <v>699</v>
       </c>
       <c r="J5" s="18" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="K5" s="18" t="s">
         <v>10</v>
@@ -5531,7 +5531,7 @@
         <v>219</v>
       </c>
       <c r="J4" s="22" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="K4" s="22" t="s">
         <v>10</v>
@@ -7814,7 +7814,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="25.5546875" customWidth="1"/>
-    <col min="4" max="4" width="35.21875" customWidth="1"/>
+    <col min="4" max="4" width="67.5546875" customWidth="1"/>
     <col min="6" max="6" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -7955,7 +7955,7 @@
         <v>1438</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="K4" s="7" t="s">
         <v>10</v>
@@ -7991,7 +7991,7 @@
         <v>1168</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>10</v>
@@ -8171,7 +8171,7 @@
         <v>1258</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="K10" s="7" t="s">
         <v>10</v>
@@ -8207,7 +8207,7 @@
         <v>1662</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="K11" s="7" t="s">
         <v>10</v>
@@ -8243,7 +8243,7 @@
         <v>2157</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="K12" s="7" t="s">
         <v>10</v>
@@ -8675,7 +8675,7 @@
         <v>880</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="K24" s="7" t="s">
         <v>10</v>
@@ -9179,7 +9179,7 @@
         <v>790</v>
       </c>
       <c r="J38" s="7" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="K38" s="8" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
bug - incorrect product addition resolved
</commit_message>
<xml_diff>
--- a/inventory/Inventory.xlsx
+++ b/inventory/Inventory.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9303"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" firstSheet="4" activeTab="6"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" firstSheet="8" activeTab="13"/>
   </bookViews>
   <sheets>
     <sheet name="Hot Wheels Mainline" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2766" uniqueCount="618">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2766" uniqueCount="616">
   <si>
     <t>Code</t>
   </si>
@@ -1117,9 +1117,6 @@
   </si>
   <si>
     <t>2016 FORD GT RACE</t>
-  </si>
-  <si>
-    <t>Hot Wheels - Treasure Hunt</t>
   </si>
   <si>
     <t>HCX99</t>
@@ -1791,9 +1788,6 @@
     <t>Ferrari 512 TR (Black)</t>
   </si>
   <si>
-    <t>Tomica Premium</t>
-  </si>
-  <si>
     <t>TPLE12</t>
   </si>
   <si>
@@ -1839,9 +1833,6 @@
     <t>Matchbox The Movie Heroes</t>
   </si>
   <si>
-    <t>Matchbox - The Movie</t>
-  </si>
-  <si>
     <t>JJP36</t>
   </si>
   <si>
@@ -1894,6 +1885,9 @@
   </si>
   <si>
     <t>Matchbox Card</t>
+  </si>
+  <si>
+    <t>Hot Wheels Silver Series</t>
   </si>
 </sst>
 </file>
@@ -4169,16 +4163,16 @@
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53" s="18" t="s">
+        <v>369</v>
+      </c>
+      <c r="B53" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C53" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D53" s="18" t="s">
         <v>370</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C53" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D53" s="18" t="s">
-        <v>371</v>
       </c>
       <c r="E53" s="3" t="s">
         <v>203</v>
@@ -4204,16 +4198,16 @@
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54" s="18" t="s">
+        <v>369</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C54" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D54" s="18" t="s">
         <v>370</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C54" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D54" s="18" t="s">
-        <v>371</v>
       </c>
       <c r="E54" s="3" t="s">
         <v>203</v>
@@ -4239,16 +4233,16 @@
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" s="18" t="s">
+        <v>371</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C55" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D55" s="18" t="s">
         <v>372</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C55" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D55" s="18" t="s">
-        <v>373</v>
       </c>
       <c r="E55" s="3" t="s">
         <v>203</v>
@@ -4274,16 +4268,16 @@
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56" s="18" t="s">
+        <v>373</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C56" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D56" s="18" t="s">
         <v>374</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C56" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D56" s="18" t="s">
-        <v>375</v>
       </c>
       <c r="E56" s="3" t="s">
         <v>203</v>
@@ -4344,16 +4338,16 @@
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58" s="18" t="s">
+        <v>377</v>
+      </c>
+      <c r="B58" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C58" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D58" s="18" t="s">
         <v>378</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C58" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D58" s="18" t="s">
-        <v>379</v>
       </c>
       <c r="E58" s="3" t="s">
         <v>203</v>
@@ -4379,16 +4373,16 @@
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59" s="18" t="s">
+        <v>379</v>
+      </c>
+      <c r="B59" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C59" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D59" s="18" t="s">
         <v>380</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C59" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D59" s="18" t="s">
-        <v>381</v>
       </c>
       <c r="E59" s="3" t="s">
         <v>203</v>
@@ -4414,16 +4408,16 @@
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="B60" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C60" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D60" s="18" t="s">
         <v>386</v>
-      </c>
-      <c r="B60" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C60" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D60" s="18" t="s">
-        <v>387</v>
       </c>
       <c r="E60" s="3" t="s">
         <v>203</v>
@@ -4458,7 +4452,7 @@
         <v>12</v>
       </c>
       <c r="D61" s="18" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="E61" s="3" t="s">
         <v>203</v>
@@ -4484,16 +4478,16 @@
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A62" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C62" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D62" s="18" t="s">
         <v>389</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C62" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D62" s="18" t="s">
-        <v>390</v>
       </c>
       <c r="E62" s="3" t="s">
         <v>203</v>
@@ -4519,16 +4513,16 @@
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A63" s="18" t="s">
+        <v>410</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C63" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D63" s="18" t="s">
         <v>411</v>
-      </c>
-      <c r="B63" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C63" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D63" s="18" t="s">
-        <v>412</v>
       </c>
       <c r="E63" s="3" t="s">
         <v>203</v>
@@ -4554,16 +4548,16 @@
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A64" s="18" t="s">
+        <v>412</v>
+      </c>
+      <c r="B64" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C64" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D64" s="23" t="s">
         <v>413</v>
-      </c>
-      <c r="B64" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C64" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D64" s="23" t="s">
-        <v>414</v>
       </c>
       <c r="E64" s="3" t="s">
         <v>203</v>
@@ -4589,16 +4583,16 @@
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A65" s="18" t="s">
+        <v>414</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C65" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D65" s="18" t="s">
         <v>415</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C65" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D65" s="18" t="s">
-        <v>416</v>
       </c>
       <c r="E65" s="3" t="s">
         <v>203</v>
@@ -4624,16 +4618,16 @@
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A66" s="18" t="s">
+        <v>416</v>
+      </c>
+      <c r="B66" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C66" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D66" s="18" t="s">
         <v>417</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C66" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D66" s="18" t="s">
-        <v>418</v>
       </c>
       <c r="E66" s="3" t="s">
         <v>203</v>
@@ -4659,16 +4653,16 @@
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A67" s="18" t="s">
+        <v>418</v>
+      </c>
+      <c r="B67" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C67" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D67" s="18" t="s">
         <v>419</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C67" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D67" s="18" t="s">
-        <v>420</v>
       </c>
       <c r="E67" s="3" t="s">
         <v>203</v>
@@ -4694,16 +4688,16 @@
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A68" s="18" t="s">
+        <v>420</v>
+      </c>
+      <c r="B68" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C68" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D68" s="18" t="s">
         <v>421</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C68" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D68" s="18" t="s">
-        <v>422</v>
       </c>
       <c r="E68" s="3" t="s">
         <v>203</v>
@@ -4729,7 +4723,7 @@
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A69" s="18" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>128</v>
@@ -4738,7 +4732,7 @@
         <v>12</v>
       </c>
       <c r="D69" s="18" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="E69" s="3" t="s">
         <v>203</v>
@@ -4764,16 +4758,16 @@
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A70" s="18" t="s">
+        <v>423</v>
+      </c>
+      <c r="B70" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C70" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D70" s="18" t="s">
         <v>424</v>
-      </c>
-      <c r="B70" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C70" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D70" s="18" t="s">
-        <v>425</v>
       </c>
       <c r="E70" s="3" t="s">
         <v>203</v>
@@ -4799,16 +4793,16 @@
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A71" s="18" t="s">
+        <v>425</v>
+      </c>
+      <c r="B71" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C71" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D71" s="18" t="s">
         <v>426</v>
-      </c>
-      <c r="B71" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C71" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D71" s="18" t="s">
-        <v>427</v>
       </c>
       <c r="E71" s="3" t="s">
         <v>203</v>
@@ -4834,16 +4828,16 @@
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A72" s="24" t="s">
+        <v>427</v>
+      </c>
+      <c r="B72" t="s">
+        <v>128</v>
+      </c>
+      <c r="C72" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D72" s="25" t="s">
         <v>428</v>
-      </c>
-      <c r="B72" t="s">
-        <v>128</v>
-      </c>
-      <c r="C72" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D72" s="25" t="s">
-        <v>429</v>
       </c>
       <c r="E72" s="3" t="s">
         <v>203</v>
@@ -4869,16 +4863,16 @@
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A73" s="24" t="s">
+        <v>429</v>
+      </c>
+      <c r="B73" t="s">
+        <v>128</v>
+      </c>
+      <c r="C73" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D73" s="25" t="s">
         <v>430</v>
-      </c>
-      <c r="B73" t="s">
-        <v>128</v>
-      </c>
-      <c r="C73" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D73" s="25" t="s">
-        <v>431</v>
       </c>
       <c r="E73" s="3" t="s">
         <v>203</v>
@@ -4904,16 +4898,16 @@
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A74" s="24" t="s">
+        <v>431</v>
+      </c>
+      <c r="B74" t="s">
+        <v>128</v>
+      </c>
+      <c r="C74" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D74" s="25" t="s">
         <v>432</v>
-      </c>
-      <c r="B74" t="s">
-        <v>128</v>
-      </c>
-      <c r="C74" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D74" s="25" t="s">
-        <v>433</v>
       </c>
       <c r="E74" s="3" t="s">
         <v>203</v>
@@ -4974,16 +4968,16 @@
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A76" s="24" t="s">
+        <v>433</v>
+      </c>
+      <c r="B76" t="s">
+        <v>128</v>
+      </c>
+      <c r="C76" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D76" s="25" t="s">
         <v>434</v>
-      </c>
-      <c r="B76" t="s">
-        <v>128</v>
-      </c>
-      <c r="C76" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D76" s="25" t="s">
-        <v>435</v>
       </c>
       <c r="E76" s="3" t="s">
         <v>203</v>
@@ -5009,16 +5003,16 @@
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A77" s="24" t="s">
+        <v>435</v>
+      </c>
+      <c r="B77" t="s">
+        <v>128</v>
+      </c>
+      <c r="C77" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D77" s="25" t="s">
         <v>436</v>
-      </c>
-      <c r="B77" t="s">
-        <v>128</v>
-      </c>
-      <c r="C77" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D77" s="25" t="s">
-        <v>437</v>
       </c>
       <c r="E77" s="3" t="s">
         <v>203</v>
@@ -5044,16 +5038,16 @@
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A78" s="24" t="s">
+        <v>437</v>
+      </c>
+      <c r="B78" t="s">
+        <v>128</v>
+      </c>
+      <c r="C78" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D78" s="25" t="s">
         <v>438</v>
-      </c>
-      <c r="B78" t="s">
-        <v>128</v>
-      </c>
-      <c r="C78" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D78" s="25" t="s">
-        <v>439</v>
       </c>
       <c r="E78" s="3" t="s">
         <v>203</v>
@@ -5079,7 +5073,7 @@
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A79" s="24" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B79" t="s">
         <v>128</v>
@@ -5114,16 +5108,16 @@
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A80" s="24" t="s">
+        <v>440</v>
+      </c>
+      <c r="B80" t="s">
+        <v>128</v>
+      </c>
+      <c r="C80" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D80" s="25" t="s">
         <v>441</v>
-      </c>
-      <c r="B80" t="s">
-        <v>128</v>
-      </c>
-      <c r="C80" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D80" s="25" t="s">
-        <v>442</v>
       </c>
       <c r="E80" s="3" t="s">
         <v>203</v>
@@ -5149,16 +5143,16 @@
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A81" s="24" t="s">
+        <v>442</v>
+      </c>
+      <c r="B81" t="s">
+        <v>128</v>
+      </c>
+      <c r="C81" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D81" s="25" t="s">
         <v>443</v>
-      </c>
-      <c r="B81" t="s">
-        <v>128</v>
-      </c>
-      <c r="C81" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D81" s="25" t="s">
-        <v>444</v>
       </c>
       <c r="E81" s="3" t="s">
         <v>203</v>
@@ -5184,16 +5178,16 @@
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A82" s="24" t="s">
+        <v>444</v>
+      </c>
+      <c r="B82" t="s">
+        <v>128</v>
+      </c>
+      <c r="C82" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D82" s="25" t="s">
         <v>445</v>
-      </c>
-      <c r="B82" t="s">
-        <v>128</v>
-      </c>
-      <c r="C82" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D82" s="25" t="s">
-        <v>446</v>
       </c>
       <c r="E82" s="3" t="s">
         <v>203</v>
@@ -5219,16 +5213,16 @@
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A83" s="24" t="s">
+        <v>446</v>
+      </c>
+      <c r="B83" t="s">
+        <v>128</v>
+      </c>
+      <c r="C83" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D83" s="25" t="s">
         <v>447</v>
-      </c>
-      <c r="B83" t="s">
-        <v>128</v>
-      </c>
-      <c r="C83" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D83" s="25" t="s">
-        <v>448</v>
       </c>
       <c r="E83" s="3" t="s">
         <v>203</v>
@@ -5254,16 +5248,16 @@
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A84" s="24" t="s">
+        <v>442</v>
+      </c>
+      <c r="B84" t="s">
+        <v>128</v>
+      </c>
+      <c r="C84" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D84" s="25" t="s">
         <v>443</v>
-      </c>
-      <c r="B84" t="s">
-        <v>128</v>
-      </c>
-      <c r="C84" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D84" s="25" t="s">
-        <v>444</v>
       </c>
       <c r="E84" s="3" t="s">
         <v>203</v>
@@ -5289,16 +5283,16 @@
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A85" s="24" t="s">
+        <v>446</v>
+      </c>
+      <c r="B85" t="s">
+        <v>128</v>
+      </c>
+      <c r="C85" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D85" s="25" t="s">
         <v>447</v>
-      </c>
-      <c r="B85" t="s">
-        <v>128</v>
-      </c>
-      <c r="C85" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D85" s="25" t="s">
-        <v>448</v>
       </c>
       <c r="E85" s="3" t="s">
         <v>203</v>
@@ -5324,16 +5318,16 @@
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A86" s="24" t="s">
+        <v>448</v>
+      </c>
+      <c r="B86" t="s">
+        <v>128</v>
+      </c>
+      <c r="C86" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D86" s="25" t="s">
         <v>449</v>
-      </c>
-      <c r="B86" t="s">
-        <v>128</v>
-      </c>
-      <c r="C86" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D86" s="25" t="s">
-        <v>450</v>
       </c>
       <c r="E86" s="3" t="s">
         <v>203</v>
@@ -5359,16 +5353,16 @@
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A87" s="24" t="s">
+        <v>425</v>
+      </c>
+      <c r="B87" t="s">
+        <v>128</v>
+      </c>
+      <c r="C87" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D87" s="25" t="s">
         <v>426</v>
-      </c>
-      <c r="B87" t="s">
-        <v>128</v>
-      </c>
-      <c r="C87" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D87" s="25" t="s">
-        <v>427</v>
       </c>
       <c r="E87" s="3" t="s">
         <v>203</v>
@@ -5429,16 +5423,16 @@
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A89" s="24" t="s">
+        <v>440</v>
+      </c>
+      <c r="B89" t="s">
+        <v>128</v>
+      </c>
+      <c r="C89" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D89" s="25" t="s">
         <v>441</v>
-      </c>
-      <c r="B89" t="s">
-        <v>128</v>
-      </c>
-      <c r="C89" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D89" s="25" t="s">
-        <v>442</v>
       </c>
       <c r="E89" s="3" t="s">
         <v>203</v>
@@ -5464,16 +5458,16 @@
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A90" s="24" t="s">
+        <v>444</v>
+      </c>
+      <c r="B90" t="s">
+        <v>128</v>
+      </c>
+      <c r="C90" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D90" s="25" t="s">
         <v>445</v>
-      </c>
-      <c r="B90" t="s">
-        <v>128</v>
-      </c>
-      <c r="C90" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D90" s="25" t="s">
-        <v>446</v>
       </c>
       <c r="E90" s="3" t="s">
         <v>203</v>
@@ -5499,7 +5493,7 @@
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A91" s="24" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B91" t="s">
         <v>128</v>
@@ -5534,16 +5528,16 @@
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A92" s="24" t="s">
+        <v>456</v>
+      </c>
+      <c r="B92" t="s">
+        <v>128</v>
+      </c>
+      <c r="C92" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D92" s="25" t="s">
         <v>457</v>
-      </c>
-      <c r="B92" t="s">
-        <v>128</v>
-      </c>
-      <c r="C92" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D92" s="25" t="s">
-        <v>458</v>
       </c>
       <c r="E92" s="3" t="s">
         <v>203</v>
@@ -5569,16 +5563,16 @@
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A93" s="24" t="s">
+        <v>458</v>
+      </c>
+      <c r="B93" t="s">
+        <v>128</v>
+      </c>
+      <c r="C93" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D93" s="25" t="s">
         <v>459</v>
-      </c>
-      <c r="B93" t="s">
-        <v>128</v>
-      </c>
-      <c r="C93" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D93" s="25" t="s">
-        <v>460</v>
       </c>
       <c r="E93" s="3" t="s">
         <v>203</v>
@@ -5604,16 +5598,16 @@
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A94" s="24" t="s">
+        <v>460</v>
+      </c>
+      <c r="B94" t="s">
+        <v>128</v>
+      </c>
+      <c r="C94" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D94" s="25" t="s">
         <v>461</v>
-      </c>
-      <c r="B94" t="s">
-        <v>128</v>
-      </c>
-      <c r="C94" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D94" s="25" t="s">
-        <v>462</v>
       </c>
       <c r="E94" s="3" t="s">
         <v>203</v>
@@ -5639,16 +5633,16 @@
     </row>
     <row r="95" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A95" s="24" t="s">
+        <v>462</v>
+      </c>
+      <c r="B95" t="s">
+        <v>128</v>
+      </c>
+      <c r="C95" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D95" s="25" t="s">
         <v>463</v>
-      </c>
-      <c r="B95" t="s">
-        <v>128</v>
-      </c>
-      <c r="C95" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D95" s="25" t="s">
-        <v>464</v>
       </c>
       <c r="E95" s="3" t="s">
         <v>203</v>
@@ -5674,16 +5668,16 @@
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A96" s="24" t="s">
+        <v>464</v>
+      </c>
+      <c r="B96" t="s">
+        <v>128</v>
+      </c>
+      <c r="C96" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D96" s="25" t="s">
         <v>465</v>
-      </c>
-      <c r="B96" t="s">
-        <v>128</v>
-      </c>
-      <c r="C96" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D96" s="25" t="s">
-        <v>466</v>
       </c>
       <c r="E96" s="3" t="s">
         <v>203</v>
@@ -5709,16 +5703,16 @@
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A97" s="24" t="s">
+        <v>466</v>
+      </c>
+      <c r="B97" t="s">
+        <v>128</v>
+      </c>
+      <c r="C97" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D97" s="26" t="s">
         <v>467</v>
-      </c>
-      <c r="B97" t="s">
-        <v>128</v>
-      </c>
-      <c r="C97" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D97" s="26" t="s">
-        <v>468</v>
       </c>
       <c r="E97" s="3" t="s">
         <v>203</v>
@@ -5753,7 +5747,7 @@
         <v>12</v>
       </c>
       <c r="D98" s="25" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="E98" s="3" t="s">
         <v>203</v>
@@ -5779,16 +5773,16 @@
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A99" s="24" t="s">
+        <v>468</v>
+      </c>
+      <c r="B99" t="s">
+        <v>128</v>
+      </c>
+      <c r="C99" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D99" s="25" t="s">
         <v>469</v>
-      </c>
-      <c r="B99" t="s">
-        <v>128</v>
-      </c>
-      <c r="C99" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D99" s="25" t="s">
-        <v>470</v>
       </c>
       <c r="E99" s="3" t="s">
         <v>203</v>
@@ -5814,16 +5808,16 @@
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A100" s="24" t="s">
+        <v>425</v>
+      </c>
+      <c r="B100" t="s">
+        <v>128</v>
+      </c>
+      <c r="C100" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D100" s="24" t="s">
         <v>426</v>
-      </c>
-      <c r="B100" t="s">
-        <v>128</v>
-      </c>
-      <c r="C100" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D100" s="24" t="s">
-        <v>427</v>
       </c>
       <c r="E100" s="3" t="s">
         <v>203</v>
@@ -5849,16 +5843,16 @@
     </row>
     <row r="101" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A101" s="24" t="s">
+        <v>425</v>
+      </c>
+      <c r="B101" t="s">
+        <v>128</v>
+      </c>
+      <c r="C101" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D101" s="24" t="s">
         <v>426</v>
-      </c>
-      <c r="B101" t="s">
-        <v>128</v>
-      </c>
-      <c r="C101" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D101" s="24" t="s">
-        <v>427</v>
       </c>
       <c r="E101" s="3" t="s">
         <v>203</v>
@@ -5884,16 +5878,16 @@
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A102" s="24" t="s">
+        <v>425</v>
+      </c>
+      <c r="B102" t="s">
+        <v>128</v>
+      </c>
+      <c r="C102" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D102" s="24" t="s">
         <v>426</v>
-      </c>
-      <c r="B102" t="s">
-        <v>128</v>
-      </c>
-      <c r="C102" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D102" s="24" t="s">
-        <v>427</v>
       </c>
       <c r="E102" s="3" t="s">
         <v>203</v>
@@ -5919,16 +5913,16 @@
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A103" s="24" t="s">
+        <v>425</v>
+      </c>
+      <c r="B103" t="s">
+        <v>128</v>
+      </c>
+      <c r="C103" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D103" s="24" t="s">
         <v>426</v>
-      </c>
-      <c r="B103" t="s">
-        <v>128</v>
-      </c>
-      <c r="C103" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D103" s="24" t="s">
-        <v>427</v>
       </c>
       <c r="E103" s="3" t="s">
         <v>203</v>
@@ -5954,16 +5948,16 @@
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A104" s="24" t="s">
+        <v>470</v>
+      </c>
+      <c r="B104" t="s">
+        <v>128</v>
+      </c>
+      <c r="C104" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D104" s="25" t="s">
         <v>471</v>
-      </c>
-      <c r="B104" t="s">
-        <v>128</v>
-      </c>
-      <c r="C104" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D104" s="25" t="s">
-        <v>472</v>
       </c>
       <c r="E104" s="3" t="s">
         <v>203</v>
@@ -5989,16 +5983,16 @@
     </row>
     <row r="105" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A105" s="24" t="s">
+        <v>472</v>
+      </c>
+      <c r="B105" t="s">
+        <v>128</v>
+      </c>
+      <c r="C105" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D105" s="25" t="s">
         <v>473</v>
-      </c>
-      <c r="B105" t="s">
-        <v>128</v>
-      </c>
-      <c r="C105" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D105" s="25" t="s">
-        <v>474</v>
       </c>
       <c r="E105" s="3" t="s">
         <v>203</v>
@@ -6024,16 +6018,16 @@
     </row>
     <row r="106" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A106" s="24" t="s">
+        <v>474</v>
+      </c>
+      <c r="B106" t="s">
+        <v>128</v>
+      </c>
+      <c r="C106" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D106" s="25" t="s">
         <v>475</v>
-      </c>
-      <c r="B106" t="s">
-        <v>128</v>
-      </c>
-      <c r="C106" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D106" s="25" t="s">
-        <v>476</v>
       </c>
       <c r="E106" s="3" t="s">
         <v>203</v>
@@ -6059,16 +6053,16 @@
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A107" s="24" t="s">
+        <v>466</v>
+      </c>
+      <c r="B107" t="s">
+        <v>128</v>
+      </c>
+      <c r="C107" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D107" s="25" t="s">
         <v>467</v>
-      </c>
-      <c r="B107" t="s">
-        <v>128</v>
-      </c>
-      <c r="C107" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D107" s="25" t="s">
-        <v>468</v>
       </c>
       <c r="E107" s="3" t="s">
         <v>203</v>
@@ -6094,16 +6088,16 @@
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A108" s="24" t="s">
+        <v>476</v>
+      </c>
+      <c r="B108" t="s">
+        <v>128</v>
+      </c>
+      <c r="C108" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D108" s="25" t="s">
         <v>477</v>
-      </c>
-      <c r="B108" t="s">
-        <v>128</v>
-      </c>
-      <c r="C108" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D108" s="25" t="s">
-        <v>478</v>
       </c>
       <c r="E108" s="3" t="s">
         <v>203</v>
@@ -6129,16 +6123,16 @@
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A109" s="24" t="s">
+        <v>478</v>
+      </c>
+      <c r="B109" t="s">
+        <v>128</v>
+      </c>
+      <c r="C109" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D109" s="25" t="s">
         <v>479</v>
-      </c>
-      <c r="B109" t="s">
-        <v>128</v>
-      </c>
-      <c r="C109" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D109" s="25" t="s">
-        <v>480</v>
       </c>
       <c r="E109" s="3" t="s">
         <v>203</v>
@@ -6164,16 +6158,16 @@
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A110" s="24" t="s">
+        <v>480</v>
+      </c>
+      <c r="B110" t="s">
+        <v>128</v>
+      </c>
+      <c r="C110" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D110" s="3" t="s">
         <v>481</v>
-      </c>
-      <c r="B110" t="s">
-        <v>128</v>
-      </c>
-      <c r="C110" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D110" s="3" t="s">
-        <v>482</v>
       </c>
       <c r="E110" s="3" t="s">
         <v>203</v>
@@ -6199,16 +6193,16 @@
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A111" s="24" t="s">
+        <v>482</v>
+      </c>
+      <c r="B111" t="s">
+        <v>128</v>
+      </c>
+      <c r="C111" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D111" s="3" t="s">
         <v>483</v>
-      </c>
-      <c r="B111" t="s">
-        <v>128</v>
-      </c>
-      <c r="C111" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D111" s="3" t="s">
-        <v>484</v>
       </c>
       <c r="E111" s="3" t="s">
         <v>203</v>
@@ -6234,16 +6228,16 @@
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A112" s="24" t="s">
+        <v>414</v>
+      </c>
+      <c r="B112" t="s">
+        <v>128</v>
+      </c>
+      <c r="C112" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D112" s="25" t="s">
         <v>415</v>
-      </c>
-      <c r="B112" t="s">
-        <v>128</v>
-      </c>
-      <c r="C112" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D112" s="25" t="s">
-        <v>416</v>
       </c>
       <c r="E112" s="3" t="s">
         <v>203</v>
@@ -6424,7 +6418,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -6433,10 +6427,10 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="F2" s="21">
         <v>46235</v>
@@ -6460,7 +6454,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
@@ -6469,10 +6463,10 @@
         <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="F3" s="21">
         <v>46235</v>
@@ -6545,7 +6539,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -6554,10 +6548,10 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
+        <v>601</v>
+      </c>
+      <c r="E2" t="s">
         <v>604</v>
-      </c>
-      <c r="E2" t="s">
-        <v>607</v>
       </c>
       <c r="F2" s="21">
         <v>46235</v>
@@ -6580,7 +6574,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
@@ -6589,10 +6583,10 @@
         <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="E3" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="F3" s="21">
         <v>46235</v>
@@ -6668,7 +6662,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -6677,10 +6671,10 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
       <c r="E2" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="F2" s="21">
         <v>46235</v>
@@ -6703,7 +6697,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
@@ -6712,10 +6706,10 @@
         <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="E3" t="s">
-        <v>599</v>
+        <v>607</v>
       </c>
       <c r="F3" s="21">
         <v>46296</v>
@@ -6733,12 +6727,12 @@
         <v>11</v>
       </c>
       <c r="K3" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
@@ -6747,10 +6741,10 @@
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="E4" t="s">
-        <v>599</v>
+        <v>607</v>
       </c>
       <c r="F4" s="21">
         <v>46296</v>
@@ -6768,12 +6762,12 @@
         <v>11</v>
       </c>
       <c r="K4" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -6782,10 +6776,10 @@
         <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="E5" t="s">
-        <v>599</v>
+        <v>607</v>
       </c>
       <c r="F5" s="21">
         <v>46296</v>
@@ -6803,7 +6797,7 @@
         <v>11</v>
       </c>
       <c r="K5" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
     </row>
   </sheetData>
@@ -6910,19 +6904,19 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="B2" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C2" t="s">
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="E2" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F2" s="21">
         <v>46266</v>
@@ -6945,19 +6939,19 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="B3" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="E3" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F3" s="21">
         <v>46266</v>
@@ -6980,19 +6974,19 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="B4" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C4" t="s">
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="E4" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F4" s="21">
         <v>46266</v>
@@ -7015,19 +7009,19 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="B5" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C5" t="s">
         <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="E5" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F5" s="21">
         <v>46266</v>
@@ -7050,19 +7044,19 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>579</v>
+      </c>
+      <c r="B6" t="s">
         <v>580</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s">
         <v>581</v>
       </c>
-      <c r="C6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" t="s">
-        <v>582</v>
-      </c>
       <c r="E6" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F6" s="21">
         <v>46296</v>
@@ -7085,19 +7079,19 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>579</v>
+      </c>
+      <c r="B7" t="s">
         <v>580</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
         <v>581</v>
       </c>
-      <c r="C7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" t="s">
-        <v>582</v>
-      </c>
       <c r="E7" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F7" s="21">
         <v>46296</v>
@@ -7120,19 +7114,19 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B8" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C8" t="s">
         <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E8" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F8" s="21">
         <v>46296</v>
@@ -7155,19 +7149,19 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="B9" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C9" t="s">
         <v>12</v>
       </c>
       <c r="D9" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E9" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F9" s="21">
         <v>46296</v>
@@ -7190,19 +7184,19 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B10" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C10" t="s">
         <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="E10" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F10" s="21">
         <v>46296</v>
@@ -7225,19 +7219,19 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B11" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C11" t="s">
         <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="E11" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F11" s="21">
         <v>46296</v>
@@ -7260,19 +7254,19 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B12" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C12" t="s">
         <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="E12" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F12" s="21">
         <v>46296</v>
@@ -7295,19 +7289,19 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="B13" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C13" t="s">
         <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="E13" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F13" s="21">
         <v>46296</v>
@@ -7330,19 +7324,19 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="B14" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C14" t="s">
         <v>12</v>
       </c>
       <c r="D14" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="E14" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F14" s="21">
         <v>46296</v>
@@ -7365,19 +7359,19 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="B15" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="C15" t="s">
         <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="E15" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="F15" s="21">
         <v>46296</v>
@@ -9014,16 +9008,16 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
+        <v>390</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="19" t="s">
         <v>391</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="19" t="s">
-        <v>392</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>190</v>
@@ -9049,16 +9043,16 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="19" t="s">
+        <v>392</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="19" t="s">
         <v>393</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="19" t="s">
-        <v>394</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>190</v>
@@ -9084,16 +9078,16 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
+        <v>394</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="19" t="s">
         <v>395</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="19" t="s">
-        <v>396</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>190</v>
@@ -9119,16 +9113,16 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
+        <v>396</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="20" t="s">
         <v>397</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="20" t="s">
-        <v>398</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>190</v>
@@ -9154,16 +9148,16 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="19" t="s">
+        <v>398</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="19" t="s">
         <v>399</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="19" t="s">
-        <v>400</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>190</v>
@@ -9189,16 +9183,16 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" s="19" t="s">
+        <v>400</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="19" t="s">
         <v>401</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="19" t="s">
-        <v>402</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>190</v>
@@ -9224,16 +9218,16 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="19" t="s">
+        <v>402</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="19" t="s">
         <v>403</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" s="19" t="s">
-        <v>404</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>190</v>
@@ -9259,16 +9253,16 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="19" t="s">
+        <v>404</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C12" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="19" t="s">
         <v>405</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" s="19" t="s">
-        <v>406</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>190</v>
@@ -9294,16 +9288,16 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="19" t="s">
+        <v>406</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="19" t="s">
         <v>407</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" s="19" t="s">
-        <v>408</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>190</v>
@@ -9329,16 +9323,16 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="19" t="s">
+        <v>408</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C14" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="19" t="s">
         <v>409</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D14" s="19" t="s">
-        <v>410</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>190</v>
@@ -9364,16 +9358,16 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="28" t="s">
+        <v>493</v>
+      </c>
+      <c r="B15" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="28" t="s">
         <v>494</v>
-      </c>
-      <c r="B15" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C15" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D15" s="28" t="s">
-        <v>495</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>190</v>
@@ -9399,16 +9393,16 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="28" t="s">
+        <v>493</v>
+      </c>
+      <c r="B16" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C16" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="28" t="s">
         <v>494</v>
-      </c>
-      <c r="B16" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C16" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" s="28" t="s">
-        <v>495</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>190</v>
@@ -9434,16 +9428,16 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="28" t="s">
+        <v>495</v>
+      </c>
+      <c r="B17" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="28" t="s">
         <v>496</v>
-      </c>
-      <c r="B17" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C17" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" s="28" t="s">
-        <v>497</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>190</v>
@@ -9469,16 +9463,16 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="28" t="s">
+        <v>495</v>
+      </c>
+      <c r="B18" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="28" t="s">
         <v>496</v>
-      </c>
-      <c r="B18" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D18" s="28" t="s">
-        <v>497</v>
       </c>
       <c r="E18" s="3" t="s">
         <v>190</v>
@@ -9504,16 +9498,16 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="28" t="s">
+        <v>497</v>
+      </c>
+      <c r="B19" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="28" t="s">
         <v>498</v>
-      </c>
-      <c r="B19" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C19" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="28" t="s">
-        <v>499</v>
       </c>
       <c r="E19" s="3" t="s">
         <v>190</v>
@@ -9539,16 +9533,16 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="28" t="s">
+        <v>497</v>
+      </c>
+      <c r="B20" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="28" t="s">
         <v>498</v>
-      </c>
-      <c r="B20" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D20" s="28" t="s">
-        <v>499</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>190</v>
@@ -9574,16 +9568,16 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="28" t="s">
+        <v>499</v>
+      </c>
+      <c r="B21" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>500</v>
-      </c>
-      <c r="B21" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C21" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>501</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>190</v>
@@ -9609,16 +9603,16 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="28" t="s">
+        <v>499</v>
+      </c>
+      <c r="B22" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>500</v>
-      </c>
-      <c r="B22" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C22" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>501</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>190</v>
@@ -9644,16 +9638,16 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="28" t="s">
+        <v>501</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="28" t="s">
         <v>502</v>
-      </c>
-      <c r="B23" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C23" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D23" s="28" t="s">
-        <v>503</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>190</v>
@@ -9679,16 +9673,16 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="28" t="s">
+        <v>501</v>
+      </c>
+      <c r="B24" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="28" t="s">
         <v>502</v>
-      </c>
-      <c r="B24" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C24" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D24" s="28" t="s">
-        <v>503</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>190</v>
@@ -9714,16 +9708,16 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="28" t="s">
+        <v>503</v>
+      </c>
+      <c r="B25" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="28" t="s">
         <v>504</v>
-      </c>
-      <c r="B25" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C25" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D25" s="28" t="s">
-        <v>505</v>
       </c>
       <c r="E25" s="3" t="s">
         <v>190</v>
@@ -9749,16 +9743,16 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="28" t="s">
+        <v>505</v>
+      </c>
+      <c r="B26" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="28" t="s">
         <v>506</v>
-      </c>
-      <c r="B26" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C26" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D26" s="28" t="s">
-        <v>507</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>190</v>
@@ -9848,7 +9842,7 @@
         <v>192</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>190</v>
+        <v>615</v>
       </c>
       <c r="F2" s="4">
         <v>46054</v>
@@ -9871,19 +9865,19 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
+        <v>381</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="19" t="s">
         <v>382</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C3" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="19" t="s">
-        <v>383</v>
-      </c>
       <c r="E3" s="3" t="s">
-        <v>190</v>
+        <v>615</v>
       </c>
       <c r="F3" s="27">
         <v>46204</v>
@@ -9906,19 +9900,19 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
+        <v>383</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C4" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" s="20" t="s">
         <v>384</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C4" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="20" t="s">
-        <v>385</v>
-      </c>
       <c r="E4" s="3" t="s">
-        <v>190</v>
+        <v>615</v>
       </c>
       <c r="F4" s="27">
         <v>46204</v>
@@ -9941,19 +9935,19 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="28" t="s">
+        <v>450</v>
+      </c>
+      <c r="B5" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C5" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="28" t="s">
         <v>451</v>
       </c>
-      <c r="B5" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="28" t="s">
-        <v>452</v>
-      </c>
       <c r="E5" s="3" t="s">
-        <v>190</v>
+        <v>615</v>
       </c>
       <c r="F5" s="4">
         <v>46235</v>
@@ -9976,19 +9970,19 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="28" t="s">
+        <v>452</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C6" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="28" t="s">
         <v>453</v>
       </c>
-      <c r="B6" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="28" t="s">
-        <v>454</v>
-      </c>
       <c r="E6" s="3" t="s">
-        <v>190</v>
+        <v>615</v>
       </c>
       <c r="F6" s="4">
         <v>46235</v>
@@ -10011,19 +10005,19 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="28" t="s">
+        <v>454</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="28" t="s">
         <v>455</v>
       </c>
-      <c r="B7" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="28" t="s">
-        <v>456</v>
-      </c>
       <c r="E7" s="3" t="s">
-        <v>190</v>
+        <v>615</v>
       </c>
       <c r="F7" s="4">
         <v>46235</v>
@@ -10046,19 +10040,19 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="28" t="s">
+        <v>484</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="28" t="s">
         <v>485</v>
       </c>
-      <c r="B8" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="28" t="s">
-        <v>486</v>
-      </c>
       <c r="E8" s="3" t="s">
-        <v>190</v>
+        <v>615</v>
       </c>
       <c r="F8" s="4">
         <v>46266</v>
@@ -10081,19 +10075,19 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="28" t="s">
+        <v>486</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>487</v>
       </c>
-      <c r="B9" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>488</v>
-      </c>
       <c r="E9" s="3" t="s">
-        <v>190</v>
+        <v>615</v>
       </c>
       <c r="F9" s="4">
         <v>46266</v>
@@ -10424,8 +10418,8 @@
       <c r="D9" t="s">
         <v>362</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>363</v>
+      <c r="E9" s="13" t="s">
+        <v>204</v>
       </c>
       <c r="F9" s="21">
         <v>46204</v>
@@ -10448,19 +10442,19 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>363</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
         <v>364</v>
       </c>
-      <c r="B10" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" t="s">
-        <v>365</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>363</v>
+      <c r="E10" s="13" t="s">
+        <v>204</v>
       </c>
       <c r="F10" s="21">
         <v>46204</v>
@@ -10483,19 +10477,19 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>365</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" t="s">
         <v>366</v>
       </c>
-      <c r="B11" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" t="s">
-        <v>367</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>363</v>
+      <c r="E11" s="13" t="s">
+        <v>204</v>
       </c>
       <c r="F11" s="21">
         <v>46204</v>
@@ -10518,19 +10512,19 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>367</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" t="s">
         <v>368</v>
       </c>
-      <c r="B12" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" t="s">
-        <v>369</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>363</v>
+      <c r="E12" s="13" t="s">
+        <v>204</v>
       </c>
       <c r="F12" s="21">
         <v>46204</v>
@@ -10553,19 +10547,19 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>375</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" t="s">
         <v>376</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" t="s">
-        <v>377</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>363</v>
+      <c r="E13" s="13" t="s">
+        <v>204</v>
       </c>
       <c r="F13" s="21">
         <v>46204</v>
@@ -10599,8 +10593,8 @@
       <c r="D14" t="s">
         <v>359</v>
       </c>
-      <c r="E14" s="3" t="s">
-        <v>363</v>
+      <c r="E14" s="13" t="s">
+        <v>204</v>
       </c>
       <c r="F14" s="21">
         <v>46204</v>
@@ -10623,19 +10617,19 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="24" t="s">
+        <v>488</v>
+      </c>
+      <c r="B15" t="s">
+        <v>128</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="25" t="s">
         <v>489</v>
       </c>
-      <c r="B15" t="s">
-        <v>128</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D15" s="25" t="s">
-        <v>490</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>363</v>
+      <c r="E15" s="13" t="s">
+        <v>204</v>
       </c>
       <c r="F15" s="4">
         <v>46266</v>
@@ -10744,7 +10738,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
       <c r="B3" t="s">
         <v>128</v>
@@ -10753,10 +10747,10 @@
         <v>12</v>
       </c>
       <c r="D3" t="s">
+        <v>508</v>
+      </c>
+      <c r="E3" t="s">
         <v>509</v>
-      </c>
-      <c r="E3" t="s">
-        <v>510</v>
       </c>
       <c r="F3" s="21">
         <v>46235</v>
@@ -10834,7 +10828,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="B2" t="s">
         <v>128</v>
@@ -10843,10 +10837,10 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="E2" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="F2" s="21">
         <v>46235</v>
@@ -10869,19 +10863,19 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="28" t="s">
+        <v>490</v>
+      </c>
+      <c r="B3" s="19" t="s">
+        <v>128</v>
+      </c>
+      <c r="C3" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="28" t="s">
+        <v>507</v>
+      </c>
+      <c r="E3" t="s">
         <v>491</v>
-      </c>
-      <c r="B3" s="19" t="s">
-        <v>128</v>
-      </c>
-      <c r="C3" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="28" t="s">
-        <v>508</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>190</v>
       </c>
       <c r="F3" s="4">
         <v>46296</v>
@@ -10972,7 +10966,7 @@
         <v>57</v>
       </c>
       <c r="E2" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F2" s="21">
         <v>46174</v>
@@ -11007,7 +11001,7 @@
         <v>59</v>
       </c>
       <c r="E3" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F3" s="21">
         <v>46174</v>
@@ -11042,7 +11036,7 @@
         <v>61</v>
       </c>
       <c r="E4" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F4" s="21">
         <v>46174</v>
@@ -11077,7 +11071,7 @@
         <v>61</v>
       </c>
       <c r="E5" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F5" s="21">
         <v>46174</v>
@@ -11112,7 +11106,7 @@
         <v>63</v>
       </c>
       <c r="E6" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F6" s="21">
         <v>46174</v>
@@ -11147,7 +11141,7 @@
         <v>59</v>
       </c>
       <c r="E7" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F7" s="21">
         <v>46174</v>
@@ -11182,7 +11176,7 @@
         <v>65</v>
       </c>
       <c r="E8" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F8" s="21">
         <v>46174</v>
@@ -11217,7 +11211,7 @@
         <v>67</v>
       </c>
       <c r="E9" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F9" s="21">
         <v>46174</v>
@@ -11252,7 +11246,7 @@
         <v>69</v>
       </c>
       <c r="E10" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F10" s="21">
         <v>46174</v>
@@ -11287,7 +11281,7 @@
         <v>71</v>
       </c>
       <c r="E11" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F11" s="21">
         <v>46174</v>
@@ -11322,7 +11316,7 @@
         <v>73</v>
       </c>
       <c r="E12" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F12" s="21">
         <v>46174</v>
@@ -11357,7 +11351,7 @@
         <v>75</v>
       </c>
       <c r="E13" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F13" s="21">
         <v>46174</v>
@@ -11392,7 +11386,7 @@
         <v>77</v>
       </c>
       <c r="E14" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F14" s="21">
         <v>46174</v>
@@ -11427,7 +11421,7 @@
         <v>79</v>
       </c>
       <c r="E15" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F15" s="21">
         <v>46174</v>
@@ -11462,7 +11456,7 @@
         <v>81</v>
       </c>
       <c r="E16" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F16" s="21">
         <v>46174</v>
@@ -11497,7 +11491,7 @@
         <v>83</v>
       </c>
       <c r="E17" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F17" s="21">
         <v>46174</v>
@@ -11532,7 +11526,7 @@
         <v>85</v>
       </c>
       <c r="E18" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F18" s="21">
         <v>46174</v>
@@ -11567,7 +11561,7 @@
         <v>87</v>
       </c>
       <c r="E19" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F19" s="21">
         <v>46174</v>
@@ -11602,7 +11596,7 @@
         <v>89</v>
       </c>
       <c r="E20" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F20" s="21">
         <v>46174</v>
@@ -11637,7 +11631,7 @@
         <v>91</v>
       </c>
       <c r="E21" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F21" s="21">
         <v>46174</v>
@@ -11672,7 +11666,7 @@
         <v>93</v>
       </c>
       <c r="E22" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F22" s="21">
         <v>46174</v>
@@ -11707,7 +11701,7 @@
         <v>95</v>
       </c>
       <c r="E23" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F23" s="21">
         <v>46174</v>
@@ -11742,7 +11736,7 @@
         <v>97</v>
       </c>
       <c r="E24" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F24" s="21">
         <v>46174</v>
@@ -11777,7 +11771,7 @@
         <v>99</v>
       </c>
       <c r="E25" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F25" s="21">
         <v>46174</v>
@@ -11812,7 +11806,7 @@
         <v>312</v>
       </c>
       <c r="E26" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F26" s="22">
         <v>46204</v>
@@ -11847,7 +11841,7 @@
         <v>312</v>
       </c>
       <c r="E27" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F27" s="22">
         <v>46204</v>
@@ -11882,7 +11876,7 @@
         <v>314</v>
       </c>
       <c r="E28" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F28" s="22">
         <v>46204</v>
@@ -11917,7 +11911,7 @@
         <v>316</v>
       </c>
       <c r="E29" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F29" s="22">
         <v>46204</v>
@@ -11952,7 +11946,7 @@
         <v>318</v>
       </c>
       <c r="E30" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F30" s="22">
         <v>46204</v>
@@ -11987,7 +11981,7 @@
         <v>320</v>
       </c>
       <c r="E31" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F31" s="22">
         <v>46204</v>
@@ -12010,7 +12004,7 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="18" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B32" s="18" t="s">
         <v>9</v>
@@ -12019,10 +12013,10 @@
         <v>12</v>
       </c>
       <c r="D32" s="18" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="E32" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F32" s="22">
         <v>46204</v>
@@ -12045,7 +12039,7 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B33" t="s">
         <v>9</v>
@@ -12054,10 +12048,10 @@
         <v>12</v>
       </c>
       <c r="D33" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="E33" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F33" s="21">
         <v>46235</v>
@@ -12080,7 +12074,7 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="B34" t="s">
         <v>9</v>
@@ -12089,10 +12083,10 @@
         <v>12</v>
       </c>
       <c r="D34" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="E34" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F34" s="21">
         <v>46235</v>
@@ -12115,7 +12109,7 @@
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="B35" t="s">
         <v>9</v>
@@ -12124,10 +12118,10 @@
         <v>12</v>
       </c>
       <c r="D35" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="E35" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F35" s="21">
         <v>46235</v>
@@ -12150,7 +12144,7 @@
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="B36" t="s">
         <v>9</v>
@@ -12159,10 +12153,10 @@
         <v>12</v>
       </c>
       <c r="D36" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="E36" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F36" s="21">
         <v>46235</v>
@@ -12185,7 +12179,7 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B37" t="s">
         <v>9</v>
@@ -12194,10 +12188,10 @@
         <v>12</v>
       </c>
       <c r="D37" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="E37" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F37" s="21">
         <v>46235</v>
@@ -12220,7 +12214,7 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B38" t="s">
         <v>9</v>
@@ -12229,10 +12223,10 @@
         <v>12</v>
       </c>
       <c r="D38" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="E38" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F38" s="21">
         <v>46235</v>
@@ -12255,7 +12249,7 @@
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B39" t="s">
         <v>9</v>
@@ -12264,10 +12258,10 @@
         <v>12</v>
       </c>
       <c r="D39" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="E39" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F39" s="21">
         <v>46235</v>
@@ -12290,7 +12284,7 @@
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B40" t="s">
         <v>9</v>
@@ -12299,10 +12293,10 @@
         <v>12</v>
       </c>
       <c r="D40" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="E40" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F40" s="21">
         <v>46235</v>
@@ -12325,7 +12319,7 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="B41" t="s">
         <v>9</v>
@@ -12334,10 +12328,10 @@
         <v>12</v>
       </c>
       <c r="D41" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="E41" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F41" s="21">
         <v>46235</v>
@@ -12360,7 +12354,7 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B42" t="s">
         <v>9</v>
@@ -12369,10 +12363,10 @@
         <v>12</v>
       </c>
       <c r="D42" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="E42" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F42" s="21">
         <v>46235</v>
@@ -12395,7 +12389,7 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="B43" t="s">
         <v>9</v>
@@ -12404,10 +12398,10 @@
         <v>12</v>
       </c>
       <c r="D43" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="E43" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F43" s="21">
         <v>46235</v>
@@ -12430,7 +12424,7 @@
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B44" t="s">
         <v>9</v>
@@ -12439,10 +12433,10 @@
         <v>12</v>
       </c>
       <c r="D44" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="E44" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F44" s="21">
         <v>46235</v>
@@ -12465,7 +12459,7 @@
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B45" t="s">
         <v>9</v>
@@ -12474,10 +12468,10 @@
         <v>12</v>
       </c>
       <c r="D45" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="E45" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F45" s="21">
         <v>46235</v>
@@ -12500,7 +12494,7 @@
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B46" t="s">
         <v>9</v>
@@ -12509,10 +12503,10 @@
         <v>12</v>
       </c>
       <c r="D46" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="E46" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F46" s="21">
         <v>46235</v>
@@ -12535,7 +12529,7 @@
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B47" t="s">
         <v>9</v>
@@ -12544,10 +12538,10 @@
         <v>12</v>
       </c>
       <c r="D47" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="E47" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F47" s="21">
         <v>46235</v>
@@ -12570,7 +12564,7 @@
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B48" t="s">
         <v>9</v>
@@ -12579,10 +12573,10 @@
         <v>12</v>
       </c>
       <c r="D48" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="E48" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F48" s="21">
         <v>46235</v>
@@ -12614,10 +12608,10 @@
         <v>12</v>
       </c>
       <c r="D49" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="E49" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F49" s="21">
         <v>46235</v>
@@ -12640,7 +12634,7 @@
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B50" t="s">
         <v>9</v>
@@ -12649,10 +12643,10 @@
         <v>12</v>
       </c>
       <c r="D50" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="E50" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F50" s="21">
         <v>46235</v>
@@ -12675,7 +12669,7 @@
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B51" t="s">
         <v>9</v>
@@ -12684,10 +12678,10 @@
         <v>12</v>
       </c>
       <c r="D51" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="E51" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F51" s="21">
         <v>46235</v>
@@ -12710,7 +12704,7 @@
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="B52" t="s">
         <v>9</v>
@@ -12719,10 +12713,10 @@
         <v>12</v>
       </c>
       <c r="D52" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="E52" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F52" s="21">
         <v>46235</v>
@@ -12745,7 +12739,7 @@
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="B53" t="s">
         <v>9</v>
@@ -12754,10 +12748,10 @@
         <v>12</v>
       </c>
       <c r="D53" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="E53" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F53" s="21">
         <v>46235</v>
@@ -12780,7 +12774,7 @@
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="B54" t="s">
         <v>9</v>
@@ -12789,10 +12783,10 @@
         <v>12</v>
       </c>
       <c r="D54" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="E54" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F54" s="21">
         <v>46266</v>
@@ -12815,7 +12809,7 @@
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="B55" t="s">
         <v>9</v>
@@ -12824,10 +12818,10 @@
         <v>12</v>
       </c>
       <c r="D55" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="E55" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F55" s="21">
         <v>46266</v>
@@ -12850,7 +12844,7 @@
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="B56" t="s">
         <v>9</v>
@@ -12859,10 +12853,10 @@
         <v>12</v>
       </c>
       <c r="D56" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="E56" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F56" s="21">
         <v>46266</v>
@@ -12885,7 +12879,7 @@
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="B57" t="s">
         <v>9</v>
@@ -12894,10 +12888,10 @@
         <v>12</v>
       </c>
       <c r="D57" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="E57" t="s">
-        <v>617</v>
+        <v>614</v>
       </c>
       <c r="F57" s="21">
         <v>46266</v>
@@ -14276,7 +14270,7 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="19" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="B16" s="19" t="s">
         <v>9</v>
@@ -14285,7 +14279,7 @@
         <v>12</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="E16" s="19" t="s">
         <v>18</v>
@@ -14311,7 +14305,7 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" s="19" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="B17" s="19" t="s">
         <v>9</v>
@@ -14320,7 +14314,7 @@
         <v>12</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="E17" s="19" t="s">
         <v>18</v>
@@ -14346,7 +14340,7 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" s="19" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B18" s="19" t="s">
         <v>9</v>
@@ -14355,7 +14349,7 @@
         <v>12</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="E18" s="19" t="s">
         <v>18</v>
@@ -14381,7 +14375,7 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" s="19" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B19" s="19" t="s">
         <v>9</v>
@@ -14390,7 +14384,7 @@
         <v>12</v>
       </c>
       <c r="D19" s="19" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="E19" s="19" t="s">
         <v>18</v>
@@ -14416,7 +14410,7 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="19" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="B20" s="19" t="s">
         <v>9</v>
@@ -14425,7 +14419,7 @@
         <v>12</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="E20" s="19" t="s">
         <v>18</v>
@@ -14451,7 +14445,7 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="19" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="B21" s="19" t="s">
         <v>9</v>
@@ -14460,7 +14454,7 @@
         <v>12</v>
       </c>
       <c r="D21" s="19" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="E21" s="19" t="s">
         <v>18</v>
@@ -14486,7 +14480,7 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="19" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="B22" s="19" t="s">
         <v>9</v>
@@ -14495,7 +14489,7 @@
         <v>12</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="E22" s="19" t="s">
         <v>18</v>
@@ -14521,7 +14515,7 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="19" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="B23" s="19" t="s">
         <v>9</v>
@@ -14530,7 +14524,7 @@
         <v>12</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="E23" s="19" t="s">
         <v>18</v>
@@ -14556,16 +14550,16 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="19" t="s">
+        <v>565</v>
+      </c>
+      <c r="B24" s="19" t="s">
         <v>566</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="C24" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="19" t="s">
         <v>567</v>
-      </c>
-      <c r="C24" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="D24" s="19" t="s">
-        <v>568</v>
       </c>
       <c r="E24" s="19" t="s">
         <v>18</v>
@@ -14586,21 +14580,21 @@
         <v>11</v>
       </c>
       <c r="K24" s="19" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="19" t="s">
+        <v>568</v>
+      </c>
+      <c r="B25" s="19" t="s">
+        <v>566</v>
+      </c>
+      <c r="C25" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="19" t="s">
         <v>569</v>
-      </c>
-      <c r="B25" s="19" t="s">
-        <v>567</v>
-      </c>
-      <c r="C25" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="D25" s="19" t="s">
-        <v>570</v>
       </c>
       <c r="E25" s="19" t="s">
         <v>18</v>
@@ -14621,21 +14615,21 @@
         <v>11</v>
       </c>
       <c r="K25" s="19" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="19" t="s">
+        <v>570</v>
+      </c>
+      <c r="B26" s="19" t="s">
+        <v>566</v>
+      </c>
+      <c r="C26" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="19" t="s">
         <v>571</v>
-      </c>
-      <c r="B26" s="19" t="s">
-        <v>567</v>
-      </c>
-      <c r="C26" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="D26" s="19" t="s">
-        <v>572</v>
       </c>
       <c r="E26" s="19" t="s">
         <v>18</v>
@@ -14656,21 +14650,21 @@
         <v>11</v>
       </c>
       <c r="K26" s="19" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="19" t="s">
+        <v>572</v>
+      </c>
+      <c r="B27" s="19" t="s">
+        <v>566</v>
+      </c>
+      <c r="C27" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="19" t="s">
         <v>573</v>
-      </c>
-      <c r="B27" s="19" t="s">
-        <v>567</v>
-      </c>
-      <c r="C27" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="D27" s="19" t="s">
-        <v>574</v>
       </c>
       <c r="E27" s="19" t="s">
         <v>18</v>
@@ -14691,21 +14685,21 @@
         <v>11</v>
       </c>
       <c r="K27" s="19" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="19" t="s">
+        <v>574</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>566</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" s="19" t="s">
         <v>575</v>
-      </c>
-      <c r="B28" s="19" t="s">
-        <v>567</v>
-      </c>
-      <c r="C28" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="D28" s="19" t="s">
-        <v>576</v>
       </c>
       <c r="E28" s="19" t="s">
         <v>18</v>
@@ -14726,15 +14720,15 @@
         <v>11</v>
       </c>
       <c r="K28" s="19" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="19" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="C29" s="19" t="s">
         <v>12</v>
@@ -14761,21 +14755,21 @@
         <v>11</v>
       </c>
       <c r="K29" s="19" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="19" t="s">
+        <v>577</v>
+      </c>
+      <c r="B30" s="19" t="s">
+        <v>566</v>
+      </c>
+      <c r="C30" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" s="19" t="s">
         <v>578</v>
-      </c>
-      <c r="B30" s="19" t="s">
-        <v>567</v>
-      </c>
-      <c r="C30" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="D30" s="19" t="s">
-        <v>579</v>
       </c>
       <c r="E30" s="19" t="s">
         <v>18</v>
@@ -14796,21 +14790,21 @@
         <v>11</v>
       </c>
       <c r="K30" s="19" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="19" t="s">
+        <v>561</v>
+      </c>
+      <c r="B31" s="19" t="s">
+        <v>566</v>
+      </c>
+      <c r="C31" s="19" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" s="19" t="s">
         <v>562</v>
-      </c>
-      <c r="B31" s="19" t="s">
-        <v>567</v>
-      </c>
-      <c r="C31" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="D31" s="19" t="s">
-        <v>563</v>
       </c>
       <c r="E31" s="19" t="s">
         <v>18</v>
@@ -14831,7 +14825,7 @@
         <v>11</v>
       </c>
       <c r="K31" s="19" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added 54% missing images
</commit_message>
<xml_diff>
--- a/inventory/Inventory.xlsx
+++ b/inventory/Inventory.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9303"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" activeTab="4"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" firstSheet="8" activeTab="13"/>
   </bookViews>
   <sheets>
     <sheet name="Hot Wheels Mainline" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2766" uniqueCount="615">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2766" uniqueCount="614">
   <si>
     <t>Code</t>
   </si>
@@ -1807,9 +1807,6 @@
   </si>
   <si>
     <t>Lamborghini Miura P400S(Red)</t>
-  </si>
-  <si>
-    <t>K0125</t>
   </si>
   <si>
     <t>ENZO FERRARI</t>
@@ -6415,7 +6412,7 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -6424,10 +6421,10 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="F2" s="21">
         <v>46235</v>
@@ -6451,7 +6448,7 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
@@ -6460,10 +6457,10 @@
         <v>12</v>
       </c>
       <c r="D3" t="s">
+        <v>596</v>
+      </c>
+      <c r="E3" s="13" t="s">
         <v>597</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>598</v>
       </c>
       <c r="F3" s="21">
         <v>46235</v>
@@ -6536,7 +6533,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -6545,10 +6542,10 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="E2" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="F2" s="21">
         <v>46235</v>
@@ -6571,7 +6568,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
@@ -6580,10 +6577,10 @@
         <v>12</v>
       </c>
       <c r="D3" t="s">
+        <v>601</v>
+      </c>
+      <c r="E3" t="s">
         <v>602</v>
-      </c>
-      <c r="E3" t="s">
-        <v>603</v>
       </c>
       <c r="F3" s="21">
         <v>46235</v>
@@ -6659,7 +6656,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B2" t="s">
         <v>9</v>
@@ -6668,10 +6665,10 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
+        <v>604</v>
+      </c>
+      <c r="E2" t="s">
         <v>605</v>
-      </c>
-      <c r="E2" t="s">
-        <v>606</v>
       </c>
       <c r="F2" s="21">
         <v>46235</v>
@@ -6694,7 +6691,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
@@ -6703,10 +6700,10 @@
         <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="E3" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="F3" s="21">
         <v>46296</v>
@@ -6724,12 +6721,12 @@
         <v>11</v>
       </c>
       <c r="K3" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
@@ -6738,10 +6735,10 @@
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="E4" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="F4" s="21">
         <v>46296</v>
@@ -6759,12 +6756,12 @@
         <v>11</v>
       </c>
       <c r="K4" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -6773,10 +6770,10 @@
         <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="E5" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="F5" s="21">
         <v>46296</v>
@@ -6794,7 +6791,7 @@
         <v>11</v>
       </c>
       <c r="K5" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
     </row>
   </sheetData>
@@ -6901,7 +6898,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B2" t="s">
         <v>579</v>
@@ -6910,7 +6907,7 @@
         <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="E2" t="s">
         <v>579</v>
@@ -6936,7 +6933,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="B3" t="s">
         <v>579</v>
@@ -6945,7 +6942,7 @@
         <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="E3" t="s">
         <v>579</v>
@@ -6971,7 +6968,7 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B4" t="s">
         <v>579</v>
@@ -6980,7 +6977,7 @@
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E4" t="s">
         <v>579</v>
@@ -7006,7 +7003,7 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B5" t="s">
         <v>579</v>
@@ -7015,7 +7012,7 @@
         <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E5" t="s">
         <v>579</v>
@@ -9839,7 +9836,7 @@
         <v>192</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="F2" s="4">
         <v>46054</v>
@@ -9874,7 +9871,7 @@
         <v>381</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="F3" s="27">
         <v>46204</v>
@@ -9909,7 +9906,7 @@
         <v>383</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="F4" s="27">
         <v>46204</v>
@@ -9944,7 +9941,7 @@
         <v>450</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="F5" s="4">
         <v>46235</v>
@@ -9979,7 +9976,7 @@
         <v>452</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="F6" s="4">
         <v>46235</v>
@@ -10014,7 +10011,7 @@
         <v>454</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="F7" s="4">
         <v>46235</v>
@@ -10049,7 +10046,7 @@
         <v>484</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="F8" s="4">
         <v>46266</v>
@@ -10084,7 +10081,7 @@
         <v>486</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="F9" s="4">
         <v>46266</v>
@@ -10735,7 +10732,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="B3" t="s">
         <v>128</v>
@@ -10825,16 +10822,16 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>609</v>
+      </c>
+      <c r="B2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
         <v>610</v>
-      </c>
-      <c r="B2" t="s">
-        <v>128</v>
-      </c>
-      <c r="C2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" t="s">
-        <v>611</v>
       </c>
       <c r="E2" t="s">
         <v>490</v>
@@ -10963,7 +10960,7 @@
         <v>57</v>
       </c>
       <c r="E2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F2" s="21">
         <v>46174</v>
@@ -10998,7 +10995,7 @@
         <v>59</v>
       </c>
       <c r="E3" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F3" s="21">
         <v>46174</v>
@@ -11033,7 +11030,7 @@
         <v>61</v>
       </c>
       <c r="E4" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F4" s="21">
         <v>46174</v>
@@ -11068,7 +11065,7 @@
         <v>61</v>
       </c>
       <c r="E5" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F5" s="21">
         <v>46174</v>
@@ -11103,7 +11100,7 @@
         <v>63</v>
       </c>
       <c r="E6" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F6" s="21">
         <v>46174</v>
@@ -11138,7 +11135,7 @@
         <v>59</v>
       </c>
       <c r="E7" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F7" s="21">
         <v>46174</v>
@@ -11173,7 +11170,7 @@
         <v>65</v>
       </c>
       <c r="E8" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F8" s="21">
         <v>46174</v>
@@ -11208,7 +11205,7 @@
         <v>67</v>
       </c>
       <c r="E9" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F9" s="21">
         <v>46174</v>
@@ -11243,7 +11240,7 @@
         <v>69</v>
       </c>
       <c r="E10" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F10" s="21">
         <v>46174</v>
@@ -11278,7 +11275,7 @@
         <v>71</v>
       </c>
       <c r="E11" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F11" s="21">
         <v>46174</v>
@@ -11313,7 +11310,7 @@
         <v>73</v>
       </c>
       <c r="E12" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F12" s="21">
         <v>46174</v>
@@ -11348,7 +11345,7 @@
         <v>75</v>
       </c>
       <c r="E13" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F13" s="21">
         <v>46174</v>
@@ -11383,7 +11380,7 @@
         <v>77</v>
       </c>
       <c r="E14" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F14" s="21">
         <v>46174</v>
@@ -11418,7 +11415,7 @@
         <v>79</v>
       </c>
       <c r="E15" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F15" s="21">
         <v>46174</v>
@@ -11453,7 +11450,7 @@
         <v>81</v>
       </c>
       <c r="E16" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F16" s="21">
         <v>46174</v>
@@ -11488,7 +11485,7 @@
         <v>83</v>
       </c>
       <c r="E17" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F17" s="21">
         <v>46174</v>
@@ -11523,7 +11520,7 @@
         <v>85</v>
       </c>
       <c r="E18" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F18" s="21">
         <v>46174</v>
@@ -11558,7 +11555,7 @@
         <v>87</v>
       </c>
       <c r="E19" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F19" s="21">
         <v>46174</v>
@@ -11593,7 +11590,7 @@
         <v>89</v>
       </c>
       <c r="E20" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F20" s="21">
         <v>46174</v>
@@ -11628,7 +11625,7 @@
         <v>91</v>
       </c>
       <c r="E21" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F21" s="21">
         <v>46174</v>
@@ -11663,7 +11660,7 @@
         <v>93</v>
       </c>
       <c r="E22" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F22" s="21">
         <v>46174</v>
@@ -11698,7 +11695,7 @@
         <v>95</v>
       </c>
       <c r="E23" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F23" s="21">
         <v>46174</v>
@@ -11733,7 +11730,7 @@
         <v>97</v>
       </c>
       <c r="E24" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F24" s="21">
         <v>46174</v>
@@ -11768,7 +11765,7 @@
         <v>99</v>
       </c>
       <c r="E25" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F25" s="21">
         <v>46174</v>
@@ -11803,7 +11800,7 @@
         <v>311</v>
       </c>
       <c r="E26" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F26" s="22">
         <v>46204</v>
@@ -11838,7 +11835,7 @@
         <v>311</v>
       </c>
       <c r="E27" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F27" s="22">
         <v>46204</v>
@@ -11873,7 +11870,7 @@
         <v>313</v>
       </c>
       <c r="E28" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F28" s="22">
         <v>46204</v>
@@ -11908,7 +11905,7 @@
         <v>315</v>
       </c>
       <c r="E29" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F29" s="22">
         <v>46204</v>
@@ -11943,7 +11940,7 @@
         <v>317</v>
       </c>
       <c r="E30" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F30" s="22">
         <v>46204</v>
@@ -11978,7 +11975,7 @@
         <v>319</v>
       </c>
       <c r="E31" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F31" s="22">
         <v>46204</v>
@@ -12013,7 +12010,7 @@
         <v>510</v>
       </c>
       <c r="E32" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F32" s="22">
         <v>46204</v>
@@ -12048,7 +12045,7 @@
         <v>512</v>
       </c>
       <c r="E33" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F33" s="21">
         <v>46235</v>
@@ -12083,7 +12080,7 @@
         <v>514</v>
       </c>
       <c r="E34" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F34" s="21">
         <v>46235</v>
@@ -12118,7 +12115,7 @@
         <v>516</v>
       </c>
       <c r="E35" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F35" s="21">
         <v>46235</v>
@@ -12153,7 +12150,7 @@
         <v>518</v>
       </c>
       <c r="E36" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F36" s="21">
         <v>46235</v>
@@ -12188,7 +12185,7 @@
         <v>520</v>
       </c>
       <c r="E37" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F37" s="21">
         <v>46235</v>
@@ -12223,7 +12220,7 @@
         <v>522</v>
       </c>
       <c r="E38" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F38" s="21">
         <v>46235</v>
@@ -12258,7 +12255,7 @@
         <v>512</v>
       </c>
       <c r="E39" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F39" s="21">
         <v>46235</v>
@@ -12293,7 +12290,7 @@
         <v>512</v>
       </c>
       <c r="E40" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F40" s="21">
         <v>46235</v>
@@ -12328,7 +12325,7 @@
         <v>524</v>
       </c>
       <c r="E41" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F41" s="21">
         <v>46235</v>
@@ -12363,7 +12360,7 @@
         <v>526</v>
       </c>
       <c r="E42" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F42" s="21">
         <v>46235</v>
@@ -12398,7 +12395,7 @@
         <v>528</v>
       </c>
       <c r="E43" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F43" s="21">
         <v>46235</v>
@@ -12433,7 +12430,7 @@
         <v>530</v>
       </c>
       <c r="E44" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F44" s="21">
         <v>46235</v>
@@ -12468,7 +12465,7 @@
         <v>532</v>
       </c>
       <c r="E45" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F45" s="21">
         <v>46235</v>
@@ -12503,7 +12500,7 @@
         <v>534</v>
       </c>
       <c r="E46" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F46" s="21">
         <v>46235</v>
@@ -12538,7 +12535,7 @@
         <v>536</v>
       </c>
       <c r="E47" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F47" s="21">
         <v>46235</v>
@@ -12573,7 +12570,7 @@
         <v>538</v>
       </c>
       <c r="E48" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F48" s="21">
         <v>46235</v>
@@ -12608,7 +12605,7 @@
         <v>539</v>
       </c>
       <c r="E49" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F49" s="21">
         <v>46235</v>
@@ -12643,7 +12640,7 @@
         <v>541</v>
       </c>
       <c r="E50" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F50" s="21">
         <v>46235</v>
@@ -12678,7 +12675,7 @@
         <v>543</v>
       </c>
       <c r="E51" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F51" s="21">
         <v>46235</v>
@@ -12713,7 +12710,7 @@
         <v>545</v>
       </c>
       <c r="E52" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F52" s="21">
         <v>46235</v>
@@ -12748,7 +12745,7 @@
         <v>547</v>
       </c>
       <c r="E53" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F53" s="21">
         <v>46235</v>
@@ -12783,7 +12780,7 @@
         <v>512</v>
       </c>
       <c r="E54" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F54" s="21">
         <v>46266</v>
@@ -12818,7 +12815,7 @@
         <v>526</v>
       </c>
       <c r="E55" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F55" s="21">
         <v>46266</v>
@@ -12853,7 +12850,7 @@
         <v>549</v>
       </c>
       <c r="E56" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F56" s="21">
         <v>46266</v>
@@ -12888,7 +12885,7 @@
         <v>551</v>
       </c>
       <c r="E57" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="F57" s="21">
         <v>46266</v>

</xml_diff>

<commit_message>
Move shared catalogue JS to catalogue.js
</commit_message>
<xml_diff>
--- a/inventory/Inventory.xlsx
+++ b/inventory/Inventory.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9303"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" firstSheet="8" activeTab="11"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" firstSheet="8" activeTab="13"/>
   </bookViews>
   <sheets>
     <sheet name="Hot Wheels Mainline" sheetId="1" r:id="rId1"/>
@@ -7205,7 +7205,7 @@
         <v>999</v>
       </c>
       <c r="J10" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="K10" t="s">
         <v>10</v>
@@ -7345,7 +7345,7 @@
         <v>999</v>
       </c>
       <c r="J14" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="K14" t="s">
         <v>10</v>

</xml_diff>